<commit_message>
sync: 新增道具表与物品图标(仅保留 itemType 1/2/3, 剔除 uesless=1)
</commit_message>
<xml_diff>
--- a/data-sources/技能养成相关.xlsx
+++ b/data-sources/技能养成相关.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\古荒遗迹2策划\1.表格目录\XLS表格\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\策划\1.表格目录\XLS表格\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="SkillActive" sheetId="1" r:id="rId1"/>
@@ -768,7 +768,7 @@
     <t>linshi/9</t>
   </si>
   <si>
-    <t>对自身一定范围内的敌人造成一次{0}</t>
+    <t>对自身一定范围内的敌人造成一次{0}\n当该技能100%物理伤害转火焰伤害时，还会释放火焰旋龙\n当该技能100%物理伤害转闪电伤害时，还会释放闪电旋龙\n当该技能100%物理伤害转冰冷伤害时，还会释放冰冷旋龙</t>
   </si>
   <si>
     <t>[[1111000040]]</t>
@@ -5381,60 +5381,60 @@
     <t>240|-250</t>
   </si>
   <si>
+    <t>偶尔漏电</t>
+  </si>
+  <si>
+    <t>攻击伤害击中时，有10%的几率触发10级[电圈]</t>
+  </si>
+  <si>
+    <t>1003002|1003010</t>
+  </si>
+  <si>
+    <t>0|-100</t>
+  </si>
+  <si>
+    <t>我麻了</t>
+  </si>
+  <si>
+    <t>对自身造成感电效果，攻击速度/施法速度提高50%</t>
+  </si>
+  <si>
+    <t>剑客1-天赋6</t>
+  </si>
+  <si>
+    <t>1003002|1003008</t>
+  </si>
+  <si>
+    <t>-240|-100</t>
+  </si>
+  <si>
+    <t>速度与激情</t>
+  </si>
+  <si>
+    <t>剑客1-天赋8</t>
+  </si>
+  <si>
+    <t>-240|150</t>
+  </si>
+  <si>
+    <t>脚底抹油</t>
+  </si>
+  <si>
+    <t>移动速度增加大于100%时，受到伤害额外减少5%</t>
+  </si>
+  <si>
+    <t>剑客1-天赋10</t>
+  </si>
+  <si>
+    <t>0|150</t>
+  </si>
+  <si>
     <t>唯快不破</t>
   </si>
   <si>
     <t>第一个技能获得攻击速度额外提高20%</t>
   </si>
   <si>
-    <t>1003002|1003010</t>
-  </si>
-  <si>
-    <t>0|-100</t>
-  </si>
-  <si>
-    <t>我麻了</t>
-  </si>
-  <si>
-    <t>对自身造成感电效果，攻击速度/施法速度提高50%</t>
-  </si>
-  <si>
-    <t>剑客1-天赋6</t>
-  </si>
-  <si>
-    <t>1003002|1003008</t>
-  </si>
-  <si>
-    <t>-240|-100</t>
-  </si>
-  <si>
-    <t>速度与激情</t>
-  </si>
-  <si>
-    <t>剑客1-天赋8</t>
-  </si>
-  <si>
-    <t>-240|150</t>
-  </si>
-  <si>
-    <t>脚底抹油</t>
-  </si>
-  <si>
-    <t>移动速度增加大于100%时，受到伤害额外减少5%</t>
-  </si>
-  <si>
-    <t>剑客1-天赋10</t>
-  </si>
-  <si>
-    <t>0|150</t>
-  </si>
-  <si>
-    <t>偶尔漏电</t>
-  </si>
-  <si>
-    <t>攻击伤害击中时，有10%的几率触发10级[电圈]</t>
-  </si>
-  <si>
     <t>剑客1-天赋12</t>
   </si>
   <si>
@@ -6509,22 +6509,22 @@
     <t>[[10033,0.06]]</t>
   </si>
   <si>
-    <t>生命恢复速度增加</t>
+    <t>生命恢复率增加</t>
   </si>
   <si>
     <t>talent/common_1/zhiliaosudu</t>
   </si>
   <si>
-    <t>生命恢复速度增加0.2%</t>
+    <t>生命恢复率增加0.2%</t>
   </si>
   <si>
     <t>[[10004,0.002]]</t>
   </si>
   <si>
-    <t>魔力恢复速度增加</t>
-  </si>
-  <si>
-    <t>魔力恢复速度增加0.2%</t>
+    <t>魔力恢复率增加</t>
+  </si>
+  <si>
+    <t>魔力恢复率增加0.2%</t>
   </si>
   <si>
     <t>[[10006,0.002]]</t>
@@ -6980,7 +6980,7 @@
     <t>抗性盘1-11</t>
   </si>
   <si>
-    <t>抗性注能持续时间提高{0}</t>
+    <t>抗性注能持续时间提高1%</t>
   </si>
   <si>
     <t>抗性盘2-1</t>
@@ -7576,14 +7576,14 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -9224,7 +9224,8 @@
       <c r="I4" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="49">
+      <c r="K4" s="49" cm="1">
+        <f t="array" ref="K4">_xlfn.SWITCH(E4,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L4" s="49" t="s">
@@ -9246,7 +9247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="17.25" spans="1:18">
+    <row r="5" ht="40.5" spans="1:18">
       <c r="A5" s="49">
         <v>100002</v>
       </c>
@@ -9271,7 +9272,8 @@
       <c r="I5" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="K5" s="49">
+      <c r="K5" s="49" cm="1">
+        <f t="array" ref="K5">_xlfn.SWITCH(E5,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L5" s="49" t="s">
@@ -9318,7 +9320,8 @@
       <c r="I6" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="K6" s="49">
+      <c r="K6" s="49" cm="1">
+        <f t="array" ref="K6">_xlfn.SWITCH(E6,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L6" s="49" t="s">
@@ -9365,7 +9368,8 @@
       <c r="I7" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K7" s="49">
+      <c r="K7" s="49" cm="1">
+        <f t="array" ref="K7">_xlfn.SWITCH(E7,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L7" s="49" t="s">
@@ -9414,7 +9418,7 @@
         <v>58</v>
       </c>
       <c r="K8" s="49" cm="1">
-        <f t="array" ref="K8">_xlfn.SWITCH(E8,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K8">_xlfn.SWITCH(E8,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L8" s="49" t="s">
@@ -9463,7 +9467,7 @@
         <v>58</v>
       </c>
       <c r="K9" s="49" cm="1">
-        <f t="array" ref="K9">_xlfn.SWITCH(E9,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K9">_xlfn.SWITCH(E9,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L9" s="49" t="s">
@@ -9512,7 +9516,7 @@
         <v>58</v>
       </c>
       <c r="K10" s="49" cm="1">
-        <f t="array" ref="K10">_xlfn.SWITCH(E10,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K10">_xlfn.SWITCH(E10,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L10" s="49" t="s">
@@ -9561,7 +9565,7 @@
         <v>58</v>
       </c>
       <c r="K11" s="49" cm="1">
-        <f t="array" ref="K11">_xlfn.SWITCH(E11,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K11">_xlfn.SWITCH(E11,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L11" s="49" t="s">
@@ -9610,7 +9614,7 @@
         <v>58</v>
       </c>
       <c r="K12" s="49" cm="1">
-        <f t="array" ref="K12">_xlfn.SWITCH(E12,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K12">_xlfn.SWITCH(E12,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L12" s="49" t="s">
@@ -9659,7 +9663,7 @@
         <v>58</v>
       </c>
       <c r="K13" s="49" cm="1">
-        <f t="array" ref="K13">_xlfn.SWITCH(E13,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K13">_xlfn.SWITCH(E13,1,0,2,7,3,10,4,15,5,50)</f>
         <v>0</v>
       </c>
       <c r="L13" s="49" t="s">
@@ -9708,7 +9712,7 @@
         <v>58</v>
       </c>
       <c r="K14" s="49" cm="1">
-        <f t="array" ref="K14">_xlfn.SWITCH(E14,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K14">_xlfn.SWITCH(E14,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L14" s="49" t="s">
@@ -9760,7 +9764,7 @@
         <v>58</v>
       </c>
       <c r="K15" s="49" cm="1">
-        <f t="array" ref="K15">_xlfn.SWITCH(E15,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K15">_xlfn.SWITCH(E15,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L15" s="49" t="s">
@@ -9812,7 +9816,7 @@
         <v>58</v>
       </c>
       <c r="K16" s="49" cm="1">
-        <f t="array" ref="K16">_xlfn.SWITCH(E16,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K16">_xlfn.SWITCH(E16,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L16" s="49" t="s">
@@ -9861,7 +9865,7 @@
         <v>58</v>
       </c>
       <c r="K17" s="49" cm="1">
-        <f t="array" ref="K17">_xlfn.SWITCH(E17,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K17">_xlfn.SWITCH(E17,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L17" s="49" t="s">
@@ -9906,8 +9910,8 @@
       <c r="I18" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K18" s="65" cm="1">
-        <f t="array" ref="K18">_xlfn.SWITCH(E18,1,0,2,7,3,15,4,25,5,50)</f>
+      <c r="K18" s="49" cm="1">
+        <f t="array" ref="K18">_xlfn.SWITCH(E18,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="M18" s="72" t="s">
@@ -9949,7 +9953,7 @@
         <v>58</v>
       </c>
       <c r="K19" s="49" cm="1">
-        <f t="array" ref="K19">_xlfn.SWITCH(E19,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K19">_xlfn.SWITCH(E19,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L19" s="49" t="s">
@@ -9999,8 +10003,9 @@
       <c r="I20" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K20" s="49">
-        <v>15</v>
+      <c r="K20" s="49" cm="1">
+        <f t="array" ref="K20">_xlfn.SWITCH(E20,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L20" s="49" t="s">
         <v>108</v>
@@ -10048,8 +10053,8 @@
         <v>58</v>
       </c>
       <c r="K21" s="49" cm="1">
-        <f t="array" ref="K21">_xlfn.SWITCH(E21,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K21">_xlfn.SWITCH(E21,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L21" s="49" t="s">
         <v>112</v>
@@ -10094,8 +10099,8 @@
         <v>58</v>
       </c>
       <c r="K22" s="49" cm="1">
-        <f t="array" ref="K22">_xlfn.SWITCH(E22,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K22">_xlfn.SWITCH(E22,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L22" s="49" t="s">
         <v>115</v>
@@ -10146,7 +10151,7 @@
         <v>58</v>
       </c>
       <c r="K23" s="49" cm="1">
-        <f t="array" ref="K23">_xlfn.SWITCH(E23,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K23">_xlfn.SWITCH(E23,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L23" s="49" t="s">
@@ -10198,8 +10203,8 @@
         <v>58</v>
       </c>
       <c r="K24" s="49" cm="1">
-        <f t="array" ref="K24">_xlfn.SWITCH(E24,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>25</v>
+        <f t="array" ref="K24">_xlfn.SWITCH(E24,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="L24" s="49" t="s">
         <v>123</v>
@@ -10242,9 +10247,9 @@
       <c r="I25" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K25" s="66" cm="1">
-        <f t="array" ref="K25">_xlfn.SWITCH(E25,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>25</v>
+      <c r="K25" s="49" cm="1">
+        <f t="array" ref="K25">_xlfn.SWITCH(E25,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="M25" s="72" t="s">
         <v>127</v>
@@ -10285,9 +10290,9 @@
       <c r="I26" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K26" s="65" cm="1">
-        <f t="array" ref="K26">_xlfn.SWITCH(E26,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>25</v>
+      <c r="K26" s="49" cm="1">
+        <f t="array" ref="K26">_xlfn.SWITCH(E26,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="M26" s="73" t="s">
         <v>129</v>
@@ -10325,8 +10330,8 @@
       <c r="I27" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K27" s="66" cm="1">
-        <f t="array" ref="K27">_xlfn.SWITCH(E27,1,0,2,7,3,15,4,25,5,50)</f>
+      <c r="K27" s="49" cm="1">
+        <f t="array" ref="K27">_xlfn.SWITCH(E27,1,0,2,7,3,10,4,15,5,50)</f>
         <v>50</v>
       </c>
       <c r="L27" s="49" t="s">
@@ -10368,8 +10373,8 @@
       <c r="I28" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K28" s="66" cm="1">
-        <f t="array" ref="K28">_xlfn.SWITCH(E28,1,0,2,7,3,15,4,25,5,50)</f>
+      <c r="K28" s="49" cm="1">
+        <f t="array" ref="K28">_xlfn.SWITCH(E28,1,0,2,7,3,10,4,15,5,50)</f>
         <v>50</v>
       </c>
       <c r="M28" s="72" t="s">
@@ -10402,7 +10407,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G29" s="49">
         <v>2114000020</v>
@@ -10415,8 +10420,8 @@
         <v>58</v>
       </c>
       <c r="K29" s="49" cm="1">
-        <f t="array" ref="K29">_xlfn.SWITCH(E29,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>50</v>
+        <f t="array" ref="K29">_xlfn.SWITCH(E29,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="L29" s="49" t="s">
         <v>131</v>
@@ -10445,7 +10450,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G30" s="49">
         <v>2140000040</v>
@@ -10458,8 +10463,8 @@
         <v>58</v>
       </c>
       <c r="K30" s="49" cm="1">
-        <f t="array" ref="K30">_xlfn.SWITCH(E30,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>50</v>
+        <f t="array" ref="K30">_xlfn.SWITCH(E30,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="L30" s="49" t="s">
         <v>135</v>
@@ -10488,7 +10493,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G31" s="49">
         <v>2140000050</v>
@@ -10501,8 +10506,8 @@
         <v>58</v>
       </c>
       <c r="K31" s="49" cm="1">
-        <f t="array" ref="K31">_xlfn.SWITCH(E31,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>50</v>
+        <f t="array" ref="K31">_xlfn.SWITCH(E31,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="L31" s="49" t="s">
         <v>137</v>
@@ -10531,7 +10536,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G32" s="49">
         <v>2140000060</v>
@@ -10544,8 +10549,8 @@
         <v>58</v>
       </c>
       <c r="K32" s="49" cm="1">
-        <f t="array" ref="K32">_xlfn.SWITCH(E32,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>50</v>
+        <f t="array" ref="K32">_xlfn.SWITCH(E32,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="L32" s="49" t="s">
         <v>139</v>
@@ -10574,7 +10579,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G33" s="49">
         <v>2140000070</v>
@@ -10587,8 +10592,8 @@
         <v>58</v>
       </c>
       <c r="K33" s="49" cm="1">
-        <f t="array" ref="K33">_xlfn.SWITCH(E33,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>50</v>
+        <f t="array" ref="K33">_xlfn.SWITCH(E33,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>15</v>
       </c>
       <c r="L33" s="49" t="s">
         <v>141</v>
@@ -10630,7 +10635,7 @@
         <v>58</v>
       </c>
       <c r="K34" s="49" cm="1">
-        <f t="array" ref="K34">_xlfn.SWITCH(E34,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K34">_xlfn.SWITCH(E34,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L34" s="49" t="s">
@@ -10673,7 +10678,7 @@
         <v>58</v>
       </c>
       <c r="K35" s="49" cm="1">
-        <f t="array" ref="K35">_xlfn.SWITCH(E35,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K35">_xlfn.SWITCH(E35,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L35" s="49" t="s">
@@ -10716,8 +10721,8 @@
         <v>58</v>
       </c>
       <c r="K36" s="49" cm="1">
-        <f t="array" ref="K36">_xlfn.SWITCH(E36,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K36">_xlfn.SWITCH(E36,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L36" s="49" t="s">
         <v>149</v>
@@ -10756,8 +10761,8 @@
         <v>58</v>
       </c>
       <c r="K37" s="49" cm="1">
-        <f t="array" ref="K37">_xlfn.SWITCH(E37,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K37">_xlfn.SWITCH(E37,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L37" s="49" t="s">
         <v>151</v>
@@ -10796,8 +10801,8 @@
         <v>58</v>
       </c>
       <c r="K38" s="49" cm="1">
-        <f t="array" ref="K38">_xlfn.SWITCH(E38,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K38">_xlfn.SWITCH(E38,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L38" s="49" t="s">
         <v>153</v>
@@ -10836,8 +10841,8 @@
         <v>58</v>
       </c>
       <c r="K39" s="49" cm="1">
-        <f t="array" ref="K39">_xlfn.SWITCH(E39,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K39">_xlfn.SWITCH(E39,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L39" s="49" t="s">
         <v>155</v>
@@ -10876,8 +10881,8 @@
         <v>58</v>
       </c>
       <c r="K40" s="49" cm="1">
-        <f t="array" ref="K40">_xlfn.SWITCH(E40,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K40">_xlfn.SWITCH(E40,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L40" s="49" t="s">
         <v>157</v>
@@ -10916,7 +10921,7 @@
         <v>58</v>
       </c>
       <c r="K41" s="49" cm="1">
-        <f t="array" ref="K41">_xlfn.SWITCH(E41,1,0,2,7,3,15,4,25,5,50)</f>
+        <f t="array" ref="K41">_xlfn.SWITCH(E41,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L41" s="49" t="s">
@@ -10965,8 +10970,8 @@
         <v>58</v>
       </c>
       <c r="K42" s="49" cm="1">
-        <f t="array" ref="K42">_xlfn.SWITCH(E42,1,0,2,7,3,15,4,25,5,50)</f>
-        <v>15</v>
+        <f t="array" ref="K42">_xlfn.SWITCH(E42,1,0,2,7,3,10,4,15,5,50)</f>
+        <v>10</v>
       </c>
       <c r="L42" s="49" t="s">
         <v>163</v>
@@ -11016,7 +11021,8 @@
       <c r="I43" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K43" s="49">
+      <c r="K43" s="49" cm="1">
+        <f t="array" ref="K43">_xlfn.SWITCH(E43,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L43" s="49" t="s">
@@ -11067,7 +11073,8 @@
       <c r="I44" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="K44" s="49">
+      <c r="K44" s="49" cm="1">
+        <f t="array" ref="K44">_xlfn.SWITCH(E44,1,0,2,7,3,10,4,15,5,50)</f>
         <v>7</v>
       </c>
       <c r="L44" s="49" t="s">
@@ -23262,7 +23269,7 @@
       </c>
       <c r="H260">
         <f>_xlfn.XLOOKUP(E260,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="261" spans="1:8">
@@ -23296,7 +23303,7 @@
       </c>
       <c r="H261">
         <f>_xlfn.XLOOKUP(E261,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="262" spans="1:8">
@@ -23330,7 +23337,7 @@
       </c>
       <c r="H262">
         <f>_xlfn.XLOOKUP(E262,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="263" spans="1:8">
@@ -23364,7 +23371,7 @@
       </c>
       <c r="H263">
         <f>_xlfn.XLOOKUP(E263,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="264" spans="1:8">
@@ -23398,7 +23405,7 @@
       </c>
       <c r="H264">
         <f>_xlfn.XLOOKUP(E264,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="265" spans="1:8">
@@ -23432,7 +23439,7 @@
       </c>
       <c r="H265">
         <f>_xlfn.XLOOKUP(E265,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="266" spans="1:8">
@@ -23466,7 +23473,7 @@
       </c>
       <c r="H266">
         <f>_xlfn.XLOOKUP(E266,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="267" spans="1:8">
@@ -23500,7 +23507,7 @@
       </c>
       <c r="H267">
         <f>_xlfn.XLOOKUP(E267,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="268" spans="1:8">
@@ -23534,7 +23541,7 @@
       </c>
       <c r="H268">
         <f>_xlfn.XLOOKUP(E268,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="269" spans="1:8">
@@ -23568,7 +23575,7 @@
       </c>
       <c r="H269">
         <f>_xlfn.XLOOKUP(E269,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="270" spans="1:8">
@@ -23602,7 +23609,7 @@
       </c>
       <c r="H270">
         <f>_xlfn.XLOOKUP(E270,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="271" spans="1:8">
@@ -23636,7 +23643,7 @@
       </c>
       <c r="H271">
         <f>_xlfn.XLOOKUP(E271,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="272" spans="1:8">
@@ -23670,7 +23677,7 @@
       </c>
       <c r="H272">
         <f>_xlfn.XLOOKUP(E272,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="273" spans="1:8">
@@ -23704,7 +23711,7 @@
       </c>
       <c r="H273">
         <f>_xlfn.XLOOKUP(E273,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="274" spans="1:8">
@@ -23738,7 +23745,7 @@
       </c>
       <c r="H274">
         <f>_xlfn.XLOOKUP(E274,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="275" spans="1:8">
@@ -23772,7 +23779,7 @@
       </c>
       <c r="H275">
         <f>_xlfn.XLOOKUP(E275,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="276" spans="1:8">
@@ -23806,7 +23813,7 @@
       </c>
       <c r="H276">
         <f>_xlfn.XLOOKUP(E276,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="277" spans="1:8">
@@ -23840,7 +23847,7 @@
       </c>
       <c r="H277">
         <f>_xlfn.XLOOKUP(E277,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="278" spans="1:8">
@@ -23874,7 +23881,7 @@
       </c>
       <c r="H278">
         <f>_xlfn.XLOOKUP(E278,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="279" spans="1:8">
@@ -23908,7 +23915,7 @@
       </c>
       <c r="H279">
         <f>_xlfn.XLOOKUP(E279,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="280" spans="1:8">
@@ -23942,7 +23949,7 @@
       </c>
       <c r="H280">
         <f>_xlfn.XLOOKUP(E280,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="281" spans="1:8">
@@ -23976,7 +23983,7 @@
       </c>
       <c r="H281">
         <f>_xlfn.XLOOKUP(E281,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="282" spans="1:8">
@@ -24010,7 +24017,7 @@
       </c>
       <c r="H282">
         <f>_xlfn.XLOOKUP(E282,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="283" spans="1:8">
@@ -24044,7 +24051,7 @@
       </c>
       <c r="H283">
         <f>_xlfn.XLOOKUP(E283,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="284" spans="1:8">
@@ -24078,7 +24085,7 @@
       </c>
       <c r="H284">
         <f>_xlfn.XLOOKUP(E284,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="285" spans="1:8">
@@ -24112,7 +24119,7 @@
       </c>
       <c r="H285">
         <f>_xlfn.XLOOKUP(E285,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="286" spans="1:8">
@@ -24146,7 +24153,7 @@
       </c>
       <c r="H286">
         <f>_xlfn.XLOOKUP(E286,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="287" spans="1:8">
@@ -24180,7 +24187,7 @@
       </c>
       <c r="H287">
         <f>_xlfn.XLOOKUP(E287,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="288" spans="1:8">
@@ -24214,7 +24221,7 @@
       </c>
       <c r="H288">
         <f>_xlfn.XLOOKUP(E288,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="289" spans="1:8">
@@ -24248,7 +24255,7 @@
       </c>
       <c r="H289">
         <f>_xlfn.XLOOKUP(E289,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="290" spans="1:8">
@@ -24282,7 +24289,7 @@
       </c>
       <c r="H290">
         <f>_xlfn.XLOOKUP(E290,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="291" spans="1:8">
@@ -24316,7 +24323,7 @@
       </c>
       <c r="H291">
         <f>_xlfn.XLOOKUP(E291,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="292" spans="1:8">
@@ -24350,7 +24357,7 @@
       </c>
       <c r="H292">
         <f>_xlfn.XLOOKUP(E292,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="293" spans="1:8">
@@ -24384,7 +24391,7 @@
       </c>
       <c r="H293">
         <f>_xlfn.XLOOKUP(E293,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="294" spans="1:8">
@@ -24418,7 +24425,7 @@
       </c>
       <c r="H294">
         <f>_xlfn.XLOOKUP(E294,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="295" spans="1:8">
@@ -24452,7 +24459,7 @@
       </c>
       <c r="H295">
         <f>_xlfn.XLOOKUP(E295,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="296" spans="1:8">
@@ -24486,7 +24493,7 @@
       </c>
       <c r="H296">
         <f>_xlfn.XLOOKUP(E296,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="297" spans="1:8">
@@ -24520,7 +24527,7 @@
       </c>
       <c r="H297">
         <f>_xlfn.XLOOKUP(E297,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="298" spans="1:8">
@@ -24554,7 +24561,7 @@
       </c>
       <c r="H298">
         <f>_xlfn.XLOOKUP(E298,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="299" spans="1:8">
@@ -24588,7 +24595,7 @@
       </c>
       <c r="H299">
         <f>_xlfn.XLOOKUP(E299,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="300" spans="1:8">
@@ -24622,7 +24629,7 @@
       </c>
       <c r="H300">
         <f>_xlfn.XLOOKUP(E300,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="301" spans="1:8">
@@ -24656,7 +24663,7 @@
       </c>
       <c r="H301">
         <f>_xlfn.XLOOKUP(E301,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="302" spans="1:8">
@@ -24690,7 +24697,7 @@
       </c>
       <c r="H302">
         <f>_xlfn.XLOOKUP(E302,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="303" spans="1:8">
@@ -24724,7 +24731,7 @@
       </c>
       <c r="H303">
         <f>_xlfn.XLOOKUP(E303,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="304" spans="1:8">
@@ -24758,7 +24765,7 @@
       </c>
       <c r="H304">
         <f>_xlfn.XLOOKUP(E304,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="305" spans="1:8">
@@ -24792,7 +24799,7 @@
       </c>
       <c r="H305">
         <f>_xlfn.XLOOKUP(E305,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="306" spans="1:8">
@@ -24826,7 +24833,7 @@
       </c>
       <c r="H306">
         <f>_xlfn.XLOOKUP(E306,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="307" spans="1:8">
@@ -24860,7 +24867,7 @@
       </c>
       <c r="H307">
         <f>_xlfn.XLOOKUP(E307,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="308" spans="1:8">
@@ -25430,7 +25437,7 @@
       </c>
       <c r="H324">
         <f>_xlfn.XLOOKUP(E324,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="325" spans="1:8">
@@ -25464,7 +25471,7 @@
       </c>
       <c r="H325">
         <f>_xlfn.XLOOKUP(E325,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="326" spans="1:8">
@@ -25498,7 +25505,7 @@
       </c>
       <c r="H326">
         <f>_xlfn.XLOOKUP(E326,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="327" spans="1:8">
@@ -25532,7 +25539,7 @@
       </c>
       <c r="H327">
         <f>_xlfn.XLOOKUP(E327,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="328" spans="1:8">
@@ -25566,7 +25573,7 @@
       </c>
       <c r="H328">
         <f>_xlfn.XLOOKUP(E328,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="329" spans="1:8">
@@ -25600,7 +25607,7 @@
       </c>
       <c r="H329">
         <f>_xlfn.XLOOKUP(E329,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="330" spans="1:8">
@@ -25634,7 +25641,7 @@
       </c>
       <c r="H330">
         <f>_xlfn.XLOOKUP(E330,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="331" spans="1:8">
@@ -25668,7 +25675,7 @@
       </c>
       <c r="H331">
         <f>_xlfn.XLOOKUP(E331,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="332" spans="1:8">
@@ -25702,7 +25709,7 @@
       </c>
       <c r="H332">
         <f>_xlfn.XLOOKUP(E332,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="333" spans="1:8">
@@ -25736,7 +25743,7 @@
       </c>
       <c r="H333">
         <f>_xlfn.XLOOKUP(E333,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="334" spans="1:8">
@@ -25770,7 +25777,7 @@
       </c>
       <c r="H334">
         <f>_xlfn.XLOOKUP(E334,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="335" spans="1:8">
@@ -25804,7 +25811,7 @@
       </c>
       <c r="H335">
         <f>_xlfn.XLOOKUP(E335,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="336" spans="1:8">
@@ -25838,7 +25845,7 @@
       </c>
       <c r="H336">
         <f>_xlfn.XLOOKUP(E336,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="337" spans="1:8">
@@ -25872,7 +25879,7 @@
       </c>
       <c r="H337">
         <f>_xlfn.XLOOKUP(E337,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="338" spans="1:8">
@@ -25906,7 +25913,7 @@
       </c>
       <c r="H338">
         <f>_xlfn.XLOOKUP(E338,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="339" spans="1:8">
@@ -25940,7 +25947,7 @@
       </c>
       <c r="H339">
         <f>_xlfn.XLOOKUP(E339,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="340" spans="1:8">
@@ -25974,7 +25981,7 @@
       </c>
       <c r="H340">
         <f>_xlfn.XLOOKUP(E340,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="341" spans="1:8">
@@ -26008,7 +26015,7 @@
       </c>
       <c r="H341">
         <f>_xlfn.XLOOKUP(E341,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="342" spans="1:8">
@@ -26042,7 +26049,7 @@
       </c>
       <c r="H342">
         <f>_xlfn.XLOOKUP(E342,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="343" spans="1:8">
@@ -26076,7 +26083,7 @@
       </c>
       <c r="H343">
         <f>_xlfn.XLOOKUP(E343,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="344" spans="1:8">
@@ -26110,7 +26117,7 @@
       </c>
       <c r="H344">
         <f>_xlfn.XLOOKUP(E344,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="345" spans="1:8">
@@ -26144,7 +26151,7 @@
       </c>
       <c r="H345">
         <f>_xlfn.XLOOKUP(E345,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="346" spans="1:8">
@@ -26178,7 +26185,7 @@
       </c>
       <c r="H346">
         <f>_xlfn.XLOOKUP(E346,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="347" spans="1:8">
@@ -26212,7 +26219,7 @@
       </c>
       <c r="H347">
         <f>_xlfn.XLOOKUP(E347,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="348" spans="1:8">
@@ -26246,7 +26253,7 @@
       </c>
       <c r="H348">
         <f>_xlfn.XLOOKUP(E348,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="349" spans="1:8">
@@ -26280,7 +26287,7 @@
       </c>
       <c r="H349">
         <f>_xlfn.XLOOKUP(E349,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="350" spans="1:8">
@@ -26314,7 +26321,7 @@
       </c>
       <c r="H350">
         <f>_xlfn.XLOOKUP(E350,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="351" spans="1:8">
@@ -26348,7 +26355,7 @@
       </c>
       <c r="H351">
         <f>_xlfn.XLOOKUP(E351,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="352" spans="1:8">
@@ -26382,7 +26389,7 @@
       </c>
       <c r="H352">
         <f>_xlfn.XLOOKUP(E352,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="353" spans="1:8">
@@ -26416,7 +26423,7 @@
       </c>
       <c r="H353">
         <f>_xlfn.XLOOKUP(E353,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="354" spans="1:8">
@@ -26450,7 +26457,7 @@
       </c>
       <c r="H354">
         <f>_xlfn.XLOOKUP(E354,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="355" spans="1:8">
@@ -26484,7 +26491,7 @@
       </c>
       <c r="H355">
         <f>_xlfn.XLOOKUP(E355,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="356" spans="1:8">
@@ -26518,7 +26525,7 @@
       </c>
       <c r="H356">
         <f>_xlfn.XLOOKUP(E356,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="357" spans="1:8">
@@ -26552,7 +26559,7 @@
       </c>
       <c r="H357">
         <f>_xlfn.XLOOKUP(E357,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="358" spans="1:8">
@@ -26586,7 +26593,7 @@
       </c>
       <c r="H358">
         <f>_xlfn.XLOOKUP(E358,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="359" spans="1:8">
@@ -26620,7 +26627,7 @@
       </c>
       <c r="H359">
         <f>_xlfn.XLOOKUP(E359,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="360" spans="1:8">
@@ -26654,7 +26661,7 @@
       </c>
       <c r="H360">
         <f>_xlfn.XLOOKUP(E360,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="361" spans="1:8">
@@ -26688,7 +26695,7 @@
       </c>
       <c r="H361">
         <f>_xlfn.XLOOKUP(E361,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="362" spans="1:8">
@@ -26722,7 +26729,7 @@
       </c>
       <c r="H362">
         <f>_xlfn.XLOOKUP(E362,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="363" spans="1:8">
@@ -26756,7 +26763,7 @@
       </c>
       <c r="H363">
         <f>_xlfn.XLOOKUP(E363,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="364" spans="1:8">
@@ -26790,7 +26797,7 @@
       </c>
       <c r="H364">
         <f>_xlfn.XLOOKUP(E364,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="365" spans="1:8">
@@ -26824,7 +26831,7 @@
       </c>
       <c r="H365">
         <f>_xlfn.XLOOKUP(E365,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="366" spans="1:8">
@@ -26858,7 +26865,7 @@
       </c>
       <c r="H366">
         <f>_xlfn.XLOOKUP(E366,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="367" spans="1:8">
@@ -26892,7 +26899,7 @@
       </c>
       <c r="H367">
         <f>_xlfn.XLOOKUP(E367,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="368" spans="1:8">
@@ -26926,7 +26933,7 @@
       </c>
       <c r="H368">
         <f>_xlfn.XLOOKUP(E368,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="369" spans="1:8">
@@ -26960,7 +26967,7 @@
       </c>
       <c r="H369">
         <f>_xlfn.XLOOKUP(E369,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="370" spans="1:8">
@@ -26994,7 +27001,7 @@
       </c>
       <c r="H370">
         <f>_xlfn.XLOOKUP(E370,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="371" spans="1:8">
@@ -27028,7 +27035,7 @@
       </c>
       <c r="H371">
         <f>_xlfn.XLOOKUP(E371,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="372" spans="1:8">
@@ -28130,7 +28137,7 @@
       </c>
       <c r="G404">
         <f>_xlfn.XLOOKUP(C404,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H404">
         <f>_xlfn.XLOOKUP(E404,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28164,7 +28171,7 @@
       </c>
       <c r="G405">
         <f>_xlfn.XLOOKUP(C405,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H405">
         <f>_xlfn.XLOOKUP(E405,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28198,7 +28205,7 @@
       </c>
       <c r="G406">
         <f>_xlfn.XLOOKUP(C406,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H406">
         <f>_xlfn.XLOOKUP(E406,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28232,7 +28239,7 @@
       </c>
       <c r="G407">
         <f>_xlfn.XLOOKUP(C407,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H407">
         <f>_xlfn.XLOOKUP(E407,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28266,7 +28273,7 @@
       </c>
       <c r="G408">
         <f>_xlfn.XLOOKUP(C408,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H408">
         <f>_xlfn.XLOOKUP(E408,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28300,7 +28307,7 @@
       </c>
       <c r="G409">
         <f>_xlfn.XLOOKUP(C409,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H409">
         <f>_xlfn.XLOOKUP(E409,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28334,7 +28341,7 @@
       </c>
       <c r="G410">
         <f>_xlfn.XLOOKUP(C410,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H410">
         <f>_xlfn.XLOOKUP(E410,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28368,7 +28375,7 @@
       </c>
       <c r="G411">
         <f>_xlfn.XLOOKUP(C411,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H411">
         <f>_xlfn.XLOOKUP(E411,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28402,7 +28409,7 @@
       </c>
       <c r="G412">
         <f>_xlfn.XLOOKUP(C412,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H412">
         <f>_xlfn.XLOOKUP(E412,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28436,7 +28443,7 @@
       </c>
       <c r="G413">
         <f>_xlfn.XLOOKUP(C413,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H413">
         <f>_xlfn.XLOOKUP(E413,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28470,7 +28477,7 @@
       </c>
       <c r="G414">
         <f>_xlfn.XLOOKUP(C414,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H414">
         <f>_xlfn.XLOOKUP(E414,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28504,7 +28511,7 @@
       </c>
       <c r="G415">
         <f>_xlfn.XLOOKUP(C415,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H415">
         <f>_xlfn.XLOOKUP(E415,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28538,7 +28545,7 @@
       </c>
       <c r="G416">
         <f>_xlfn.XLOOKUP(C416,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H416">
         <f>_xlfn.XLOOKUP(E416,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28572,7 +28579,7 @@
       </c>
       <c r="G417">
         <f>_xlfn.XLOOKUP(C417,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H417">
         <f>_xlfn.XLOOKUP(E417,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28606,7 +28613,7 @@
       </c>
       <c r="G418">
         <f>_xlfn.XLOOKUP(C418,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H418">
         <f>_xlfn.XLOOKUP(E418,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28640,7 +28647,7 @@
       </c>
       <c r="G419">
         <f>_xlfn.XLOOKUP(C419,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H419">
         <f>_xlfn.XLOOKUP(E419,SkillActive!B:B,SkillActive!K:K,,0)</f>
@@ -28674,11 +28681,11 @@
       </c>
       <c r="G420">
         <f>_xlfn.XLOOKUP(C420,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H420">
         <f>_xlfn.XLOOKUP(E420,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="421" spans="1:8">
@@ -28708,11 +28715,11 @@
       </c>
       <c r="G421">
         <f>_xlfn.XLOOKUP(C421,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H421">
         <f>_xlfn.XLOOKUP(E421,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="422" spans="1:8">
@@ -28742,11 +28749,11 @@
       </c>
       <c r="G422">
         <f>_xlfn.XLOOKUP(C422,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H422">
         <f>_xlfn.XLOOKUP(E422,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="423" spans="1:8">
@@ -28776,11 +28783,11 @@
       </c>
       <c r="G423">
         <f>_xlfn.XLOOKUP(C423,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H423">
         <f>_xlfn.XLOOKUP(E423,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="424" spans="1:8">
@@ -28810,11 +28817,11 @@
       </c>
       <c r="G424">
         <f>_xlfn.XLOOKUP(C424,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H424">
         <f>_xlfn.XLOOKUP(E424,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="425" spans="1:8">
@@ -28844,11 +28851,11 @@
       </c>
       <c r="G425">
         <f>_xlfn.XLOOKUP(C425,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H425">
         <f>_xlfn.XLOOKUP(E425,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="426" spans="1:8">
@@ -28878,11 +28885,11 @@
       </c>
       <c r="G426">
         <f>_xlfn.XLOOKUP(C426,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H426">
         <f>_xlfn.XLOOKUP(E426,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="427" spans="1:8">
@@ -28912,11 +28919,11 @@
       </c>
       <c r="G427">
         <f>_xlfn.XLOOKUP(C427,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H427">
         <f>_xlfn.XLOOKUP(E427,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="428" spans="1:8">
@@ -28946,11 +28953,11 @@
       </c>
       <c r="G428">
         <f>_xlfn.XLOOKUP(C428,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H428">
         <f>_xlfn.XLOOKUP(E428,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="429" spans="1:8">
@@ -28980,11 +28987,11 @@
       </c>
       <c r="G429">
         <f>_xlfn.XLOOKUP(C429,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H429">
         <f>_xlfn.XLOOKUP(E429,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="430" spans="1:8">
@@ -29014,11 +29021,11 @@
       </c>
       <c r="G430">
         <f>_xlfn.XLOOKUP(C430,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H430">
         <f>_xlfn.XLOOKUP(E430,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="431" spans="1:8">
@@ -29048,11 +29055,11 @@
       </c>
       <c r="G431">
         <f>_xlfn.XLOOKUP(C431,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H431">
         <f>_xlfn.XLOOKUP(E431,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="432" spans="1:8">
@@ -29082,11 +29089,11 @@
       </c>
       <c r="G432">
         <f>_xlfn.XLOOKUP(C432,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H432">
         <f>_xlfn.XLOOKUP(E432,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="433" spans="1:8">
@@ -29116,11 +29123,11 @@
       </c>
       <c r="G433">
         <f>_xlfn.XLOOKUP(C433,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H433">
         <f>_xlfn.XLOOKUP(E433,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="434" spans="1:8">
@@ -29150,11 +29157,11 @@
       </c>
       <c r="G434">
         <f>_xlfn.XLOOKUP(C434,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H434">
         <f>_xlfn.XLOOKUP(E434,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="435" spans="1:8">
@@ -29184,11 +29191,11 @@
       </c>
       <c r="G435">
         <f>_xlfn.XLOOKUP(C435,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H435">
         <f>_xlfn.XLOOKUP(E435,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="436" spans="1:8">
@@ -29218,11 +29225,11 @@
       </c>
       <c r="G436">
         <f>_xlfn.XLOOKUP(C436,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H436">
         <f>_xlfn.XLOOKUP(E436,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="437" spans="1:8">
@@ -29252,11 +29259,11 @@
       </c>
       <c r="G437">
         <f>_xlfn.XLOOKUP(C437,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H437">
         <f>_xlfn.XLOOKUP(E437,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="438" spans="1:8">
@@ -29286,11 +29293,11 @@
       </c>
       <c r="G438">
         <f>_xlfn.XLOOKUP(C438,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H438">
         <f>_xlfn.XLOOKUP(E438,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="439" spans="1:8">
@@ -29320,11 +29327,11 @@
       </c>
       <c r="G439">
         <f>_xlfn.XLOOKUP(C439,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H439">
         <f>_xlfn.XLOOKUP(E439,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="440" spans="1:8">
@@ -29354,11 +29361,11 @@
       </c>
       <c r="G440">
         <f>_xlfn.XLOOKUP(C440,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H440">
         <f>_xlfn.XLOOKUP(E440,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="441" spans="1:8">
@@ -29388,11 +29395,11 @@
       </c>
       <c r="G441">
         <f>_xlfn.XLOOKUP(C441,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H441">
         <f>_xlfn.XLOOKUP(E441,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="442" spans="1:8">
@@ -29422,11 +29429,11 @@
       </c>
       <c r="G442">
         <f>_xlfn.XLOOKUP(C442,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H442">
         <f>_xlfn.XLOOKUP(E442,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="443" spans="1:8">
@@ -29456,11 +29463,11 @@
       </c>
       <c r="G443">
         <f>_xlfn.XLOOKUP(C443,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H443">
         <f>_xlfn.XLOOKUP(E443,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="444" spans="1:8">
@@ -29490,11 +29497,11 @@
       </c>
       <c r="G444">
         <f>_xlfn.XLOOKUP(C444,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H444">
         <f>_xlfn.XLOOKUP(E444,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="445" spans="1:8">
@@ -29524,11 +29531,11 @@
       </c>
       <c r="G445">
         <f>_xlfn.XLOOKUP(C445,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H445">
         <f>_xlfn.XLOOKUP(E445,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="446" spans="1:8">
@@ -29558,11 +29565,11 @@
       </c>
       <c r="G446">
         <f>_xlfn.XLOOKUP(C446,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H446">
         <f>_xlfn.XLOOKUP(E446,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="447" spans="1:8">
@@ -29592,11 +29599,11 @@
       </c>
       <c r="G447">
         <f>_xlfn.XLOOKUP(C447,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H447">
         <f>_xlfn.XLOOKUP(E447,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="448" spans="1:8">
@@ -29626,11 +29633,11 @@
       </c>
       <c r="G448">
         <f>_xlfn.XLOOKUP(C448,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H448">
         <f>_xlfn.XLOOKUP(E448,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="449" spans="1:8">
@@ -29660,11 +29667,11 @@
       </c>
       <c r="G449">
         <f>_xlfn.XLOOKUP(C449,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H449">
         <f>_xlfn.XLOOKUP(E449,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="450" spans="1:8">
@@ -29694,11 +29701,11 @@
       </c>
       <c r="G450">
         <f>_xlfn.XLOOKUP(C450,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H450">
         <f>_xlfn.XLOOKUP(E450,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="451" spans="1:8">
@@ -29728,11 +29735,11 @@
       </c>
       <c r="G451">
         <f>_xlfn.XLOOKUP(C451,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H451">
         <f>_xlfn.XLOOKUP(E451,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="452" spans="1:8">
@@ -29762,11 +29769,11 @@
       </c>
       <c r="G452">
         <f>_xlfn.XLOOKUP(C452,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H452">
         <f>_xlfn.XLOOKUP(E452,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="453" spans="1:8">
@@ -29796,11 +29803,11 @@
       </c>
       <c r="G453">
         <f>_xlfn.XLOOKUP(C453,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H453">
         <f>_xlfn.XLOOKUP(E453,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="454" spans="1:8">
@@ -29830,11 +29837,11 @@
       </c>
       <c r="G454">
         <f>_xlfn.XLOOKUP(C454,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H454">
         <f>_xlfn.XLOOKUP(E454,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="455" spans="1:8">
@@ -29864,11 +29871,11 @@
       </c>
       <c r="G455">
         <f>_xlfn.XLOOKUP(C455,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H455">
         <f>_xlfn.XLOOKUP(E455,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="456" spans="1:8">
@@ -29898,11 +29905,11 @@
       </c>
       <c r="G456">
         <f>_xlfn.XLOOKUP(C456,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H456">
         <f>_xlfn.XLOOKUP(E456,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="457" spans="1:8">
@@ -29932,11 +29939,11 @@
       </c>
       <c r="G457">
         <f>_xlfn.XLOOKUP(C457,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H457">
         <f>_xlfn.XLOOKUP(E457,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="458" spans="1:8">
@@ -29966,11 +29973,11 @@
       </c>
       <c r="G458">
         <f>_xlfn.XLOOKUP(C458,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H458">
         <f>_xlfn.XLOOKUP(E458,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="459" spans="1:8">
@@ -30000,11 +30007,11 @@
       </c>
       <c r="G459">
         <f>_xlfn.XLOOKUP(C459,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H459">
         <f>_xlfn.XLOOKUP(E459,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="460" spans="1:8">
@@ -30034,11 +30041,11 @@
       </c>
       <c r="G460">
         <f>_xlfn.XLOOKUP(C460,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H460">
         <f>_xlfn.XLOOKUP(E460,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="461" spans="1:8">
@@ -30068,11 +30075,11 @@
       </c>
       <c r="G461">
         <f>_xlfn.XLOOKUP(C461,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H461">
         <f>_xlfn.XLOOKUP(E461,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="462" spans="1:8">
@@ -30102,11 +30109,11 @@
       </c>
       <c r="G462">
         <f>_xlfn.XLOOKUP(C462,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H462">
         <f>_xlfn.XLOOKUP(E462,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="463" spans="1:8">
@@ -30136,11 +30143,11 @@
       </c>
       <c r="G463">
         <f>_xlfn.XLOOKUP(C463,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H463">
         <f>_xlfn.XLOOKUP(E463,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="464" spans="1:8">
@@ -30170,11 +30177,11 @@
       </c>
       <c r="G464">
         <f>_xlfn.XLOOKUP(C464,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H464">
         <f>_xlfn.XLOOKUP(E464,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="465" spans="1:8">
@@ -30204,11 +30211,11 @@
       </c>
       <c r="G465">
         <f>_xlfn.XLOOKUP(C465,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H465">
         <f>_xlfn.XLOOKUP(E465,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="466" spans="1:8">
@@ -30238,11 +30245,11 @@
       </c>
       <c r="G466">
         <f>_xlfn.XLOOKUP(C466,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H466">
         <f>_xlfn.XLOOKUP(E466,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="467" spans="1:8">
@@ -30272,11 +30279,11 @@
       </c>
       <c r="G467">
         <f>_xlfn.XLOOKUP(C467,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H467">
         <f>_xlfn.XLOOKUP(E467,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="468" spans="1:8">
@@ -30306,11 +30313,11 @@
       </c>
       <c r="G468">
         <f>_xlfn.XLOOKUP(C468,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H468">
         <f>_xlfn.XLOOKUP(E468,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="469" spans="1:8">
@@ -30340,11 +30347,11 @@
       </c>
       <c r="G469">
         <f>_xlfn.XLOOKUP(C469,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H469">
         <f>_xlfn.XLOOKUP(E469,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="470" spans="1:8">
@@ -30374,11 +30381,11 @@
       </c>
       <c r="G470">
         <f>_xlfn.XLOOKUP(C470,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H470">
         <f>_xlfn.XLOOKUP(E470,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="471" spans="1:8">
@@ -30408,11 +30415,11 @@
       </c>
       <c r="G471">
         <f>_xlfn.XLOOKUP(C471,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H471">
         <f>_xlfn.XLOOKUP(E471,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="472" spans="1:8">
@@ -30442,11 +30449,11 @@
       </c>
       <c r="G472">
         <f>_xlfn.XLOOKUP(C472,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H472">
         <f>_xlfn.XLOOKUP(E472,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="473" spans="1:8">
@@ -30476,11 +30483,11 @@
       </c>
       <c r="G473">
         <f>_xlfn.XLOOKUP(C473,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H473">
         <f>_xlfn.XLOOKUP(E473,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="474" spans="1:8">
@@ -30510,11 +30517,11 @@
       </c>
       <c r="G474">
         <f>_xlfn.XLOOKUP(C474,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H474">
         <f>_xlfn.XLOOKUP(E474,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="475" spans="1:8">
@@ -30544,11 +30551,11 @@
       </c>
       <c r="G475">
         <f>_xlfn.XLOOKUP(C475,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H475">
         <f>_xlfn.XLOOKUP(E475,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="476" spans="1:8">
@@ -30578,11 +30585,11 @@
       </c>
       <c r="G476">
         <f>_xlfn.XLOOKUP(C476,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H476">
         <f>_xlfn.XLOOKUP(E476,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="477" spans="1:8">
@@ -30612,11 +30619,11 @@
       </c>
       <c r="G477">
         <f>_xlfn.XLOOKUP(C477,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H477">
         <f>_xlfn.XLOOKUP(E477,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="478" spans="1:8">
@@ -30646,11 +30653,11 @@
       </c>
       <c r="G478">
         <f>_xlfn.XLOOKUP(C478,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H478">
         <f>_xlfn.XLOOKUP(E478,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="479" spans="1:8">
@@ -30680,11 +30687,11 @@
       </c>
       <c r="G479">
         <f>_xlfn.XLOOKUP(C479,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H479">
         <f>_xlfn.XLOOKUP(E479,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="480" spans="1:8">
@@ -30714,11 +30721,11 @@
       </c>
       <c r="G480">
         <f>_xlfn.XLOOKUP(C480,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H480">
         <f>_xlfn.XLOOKUP(E480,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="481" spans="1:8">
@@ -30748,11 +30755,11 @@
       </c>
       <c r="G481">
         <f>_xlfn.XLOOKUP(C481,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H481">
         <f>_xlfn.XLOOKUP(E481,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="482" spans="1:8">
@@ -30782,11 +30789,11 @@
       </c>
       <c r="G482">
         <f>_xlfn.XLOOKUP(C482,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H482">
         <f>_xlfn.XLOOKUP(E482,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="483" spans="1:8">
@@ -30816,11 +30823,11 @@
       </c>
       <c r="G483">
         <f>_xlfn.XLOOKUP(C483,SkillActive!$A:$A,SkillActive!E:E,,0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H483">
         <f>_xlfn.XLOOKUP(E483,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="484" spans="1:8">
@@ -31861,7 +31868,7 @@
       </c>
       <c r="H516">
         <f>_xlfn.XLOOKUP(E516,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="517" spans="1:8">
@@ -31894,7 +31901,7 @@
       </c>
       <c r="H517">
         <f>_xlfn.XLOOKUP(E517,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="518" spans="1:8">
@@ -31927,7 +31934,7 @@
       </c>
       <c r="H518">
         <f>_xlfn.XLOOKUP(E518,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="519" spans="1:8">
@@ -31960,7 +31967,7 @@
       </c>
       <c r="H519">
         <f>_xlfn.XLOOKUP(E519,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="520" spans="1:8">
@@ -31993,7 +32000,7 @@
       </c>
       <c r="H520">
         <f>_xlfn.XLOOKUP(E520,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="521" spans="1:8">
@@ -32026,7 +32033,7 @@
       </c>
       <c r="H521">
         <f>_xlfn.XLOOKUP(E521,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="522" spans="1:8">
@@ -32059,7 +32066,7 @@
       </c>
       <c r="H522">
         <f>_xlfn.XLOOKUP(E522,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="523" spans="1:8">
@@ -32092,7 +32099,7 @@
       </c>
       <c r="H523">
         <f>_xlfn.XLOOKUP(E523,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="524" spans="1:8">
@@ -32125,7 +32132,7 @@
       </c>
       <c r="H524">
         <f>_xlfn.XLOOKUP(E524,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="525" spans="1:8">
@@ -32158,7 +32165,7 @@
       </c>
       <c r="H525">
         <f>_xlfn.XLOOKUP(E525,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="526" spans="1:8">
@@ -32191,7 +32198,7 @@
       </c>
       <c r="H526">
         <f>_xlfn.XLOOKUP(E526,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="527" spans="1:8">
@@ -32224,7 +32231,7 @@
       </c>
       <c r="H527">
         <f>_xlfn.XLOOKUP(E527,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="528" spans="1:8">
@@ -32257,7 +32264,7 @@
       </c>
       <c r="H528">
         <f>_xlfn.XLOOKUP(E528,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="529" spans="1:8">
@@ -32290,7 +32297,7 @@
       </c>
       <c r="H529">
         <f>_xlfn.XLOOKUP(E529,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="530" spans="1:8">
@@ -32323,7 +32330,7 @@
       </c>
       <c r="H530">
         <f>_xlfn.XLOOKUP(E530,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="531" spans="1:8">
@@ -32356,7 +32363,7 @@
       </c>
       <c r="H531">
         <f>_xlfn.XLOOKUP(E531,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="532" spans="1:8">
@@ -32389,7 +32396,7 @@
       </c>
       <c r="H532">
         <f>_xlfn.XLOOKUP(E532,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="533" spans="1:8">
@@ -32422,7 +32429,7 @@
       </c>
       <c r="H533">
         <f>_xlfn.XLOOKUP(E533,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="534" spans="1:8">
@@ -32455,7 +32462,7 @@
       </c>
       <c r="H534">
         <f>_xlfn.XLOOKUP(E534,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="535" spans="1:8">
@@ -32488,7 +32495,7 @@
       </c>
       <c r="H535">
         <f>_xlfn.XLOOKUP(E535,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="536" spans="1:8">
@@ -32521,7 +32528,7 @@
       </c>
       <c r="H536">
         <f>_xlfn.XLOOKUP(E536,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="537" spans="1:8">
@@ -32554,7 +32561,7 @@
       </c>
       <c r="H537">
         <f>_xlfn.XLOOKUP(E537,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="538" spans="1:8">
@@ -32587,7 +32594,7 @@
       </c>
       <c r="H538">
         <f>_xlfn.XLOOKUP(E538,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="539" spans="1:8">
@@ -32620,7 +32627,7 @@
       </c>
       <c r="H539">
         <f>_xlfn.XLOOKUP(E539,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="540" spans="1:8">
@@ -32653,7 +32660,7 @@
       </c>
       <c r="H540">
         <f>_xlfn.XLOOKUP(E540,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="541" spans="1:8">
@@ -32686,7 +32693,7 @@
       </c>
       <c r="H541">
         <f>_xlfn.XLOOKUP(E541,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="542" spans="1:8">
@@ -32719,7 +32726,7 @@
       </c>
       <c r="H542">
         <f>_xlfn.XLOOKUP(E542,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="543" spans="1:8">
@@ -32752,7 +32759,7 @@
       </c>
       <c r="H543">
         <f>_xlfn.XLOOKUP(E543,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="544" spans="1:8">
@@ -32785,7 +32792,7 @@
       </c>
       <c r="H544">
         <f>_xlfn.XLOOKUP(E544,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="545" spans="1:8">
@@ -32818,7 +32825,7 @@
       </c>
       <c r="H545">
         <f>_xlfn.XLOOKUP(E545,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="546" spans="1:8">
@@ -32851,7 +32858,7 @@
       </c>
       <c r="H546">
         <f>_xlfn.XLOOKUP(E546,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="547" spans="1:8">
@@ -32884,7 +32891,7 @@
       </c>
       <c r="H547">
         <f>_xlfn.XLOOKUP(E547,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="548" spans="1:8">
@@ -32917,7 +32924,7 @@
       </c>
       <c r="H548">
         <f>_xlfn.XLOOKUP(E548,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="549" spans="1:8">
@@ -32950,7 +32957,7 @@
       </c>
       <c r="H549">
         <f>_xlfn.XLOOKUP(E549,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="550" spans="1:8">
@@ -32983,7 +32990,7 @@
       </c>
       <c r="H550">
         <f>_xlfn.XLOOKUP(E550,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="551" spans="1:8">
@@ -33016,7 +33023,7 @@
       </c>
       <c r="H551">
         <f>_xlfn.XLOOKUP(E551,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="552" spans="1:8">
@@ -33049,7 +33056,7 @@
       </c>
       <c r="H552">
         <f>_xlfn.XLOOKUP(E552,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="553" spans="1:8">
@@ -33082,7 +33089,7 @@
       </c>
       <c r="H553">
         <f>_xlfn.XLOOKUP(E553,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="554" spans="1:8">
@@ -33115,7 +33122,7 @@
       </c>
       <c r="H554">
         <f>_xlfn.XLOOKUP(E554,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="555" spans="1:8">
@@ -33148,7 +33155,7 @@
       </c>
       <c r="H555">
         <f>_xlfn.XLOOKUP(E555,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="556" spans="1:8">
@@ -33181,7 +33188,7 @@
       </c>
       <c r="H556">
         <f>_xlfn.XLOOKUP(E556,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="557" spans="1:8">
@@ -33214,7 +33221,7 @@
       </c>
       <c r="H557">
         <f>_xlfn.XLOOKUP(E557,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="558" spans="1:8">
@@ -33247,7 +33254,7 @@
       </c>
       <c r="H558">
         <f>_xlfn.XLOOKUP(E558,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="559" spans="1:8">
@@ -33280,7 +33287,7 @@
       </c>
       <c r="H559">
         <f>_xlfn.XLOOKUP(E559,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="560" spans="1:8">
@@ -33313,7 +33320,7 @@
       </c>
       <c r="H560">
         <f>_xlfn.XLOOKUP(E560,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="561" spans="1:8">
@@ -33346,7 +33353,7 @@
       </c>
       <c r="H561">
         <f>_xlfn.XLOOKUP(E561,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="562" spans="1:8">
@@ -33379,7 +33386,7 @@
       </c>
       <c r="H562">
         <f>_xlfn.XLOOKUP(E562,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="563" spans="1:8">
@@ -33412,7 +33419,7 @@
       </c>
       <c r="H563">
         <f>_xlfn.XLOOKUP(E563,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="564" spans="1:8">
@@ -33445,7 +33452,7 @@
       </c>
       <c r="H564">
         <f>_xlfn.XLOOKUP(E564,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="565" spans="1:8">
@@ -33478,7 +33485,7 @@
       </c>
       <c r="H565">
         <f>_xlfn.XLOOKUP(E565,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="566" spans="1:8">
@@ -33511,7 +33518,7 @@
       </c>
       <c r="H566">
         <f>_xlfn.XLOOKUP(E566,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="567" spans="1:8">
@@ -33544,7 +33551,7 @@
       </c>
       <c r="H567">
         <f>_xlfn.XLOOKUP(E567,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="568" spans="1:8">
@@ -33577,7 +33584,7 @@
       </c>
       <c r="H568">
         <f>_xlfn.XLOOKUP(E568,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="569" spans="1:8">
@@ -33610,7 +33617,7 @@
       </c>
       <c r="H569">
         <f>_xlfn.XLOOKUP(E569,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="570" spans="1:8">
@@ -33643,7 +33650,7 @@
       </c>
       <c r="H570">
         <f>_xlfn.XLOOKUP(E570,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="571" spans="1:8">
@@ -33676,7 +33683,7 @@
       </c>
       <c r="H571">
         <f>_xlfn.XLOOKUP(E571,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="572" spans="1:8">
@@ -33709,7 +33716,7 @@
       </c>
       <c r="H572">
         <f>_xlfn.XLOOKUP(E572,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="573" spans="1:8">
@@ -33742,7 +33749,7 @@
       </c>
       <c r="H573">
         <f>_xlfn.XLOOKUP(E573,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="574" spans="1:8">
@@ -33775,7 +33782,7 @@
       </c>
       <c r="H574">
         <f>_xlfn.XLOOKUP(E574,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="575" spans="1:8">
@@ -33808,7 +33815,7 @@
       </c>
       <c r="H575">
         <f>_xlfn.XLOOKUP(E575,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="576" spans="1:8">
@@ -33841,7 +33848,7 @@
       </c>
       <c r="H576">
         <f>_xlfn.XLOOKUP(E576,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="577" spans="1:8">
@@ -33874,7 +33881,7 @@
       </c>
       <c r="H577">
         <f>_xlfn.XLOOKUP(E577,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="578" spans="1:8">
@@ -33907,7 +33914,7 @@
       </c>
       <c r="H578">
         <f>_xlfn.XLOOKUP(E578,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="579" spans="1:8">
@@ -33940,7 +33947,7 @@
       </c>
       <c r="H579">
         <f>_xlfn.XLOOKUP(E579,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="580" spans="1:8">
@@ -33973,7 +33980,7 @@
       </c>
       <c r="H580">
         <f>_xlfn.XLOOKUP(E580,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="581" spans="1:8">
@@ -34006,7 +34013,7 @@
       </c>
       <c r="H581">
         <f>_xlfn.XLOOKUP(E581,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="582" spans="1:8">
@@ -34039,7 +34046,7 @@
       </c>
       <c r="H582">
         <f>_xlfn.XLOOKUP(E582,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="583" spans="1:8">
@@ -34072,7 +34079,7 @@
       </c>
       <c r="H583">
         <f>_xlfn.XLOOKUP(E583,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="584" spans="1:8">
@@ -34105,7 +34112,7 @@
       </c>
       <c r="H584">
         <f>_xlfn.XLOOKUP(E584,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="585" spans="1:8">
@@ -34138,7 +34145,7 @@
       </c>
       <c r="H585">
         <f>_xlfn.XLOOKUP(E585,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="586" spans="1:8">
@@ -34171,7 +34178,7 @@
       </c>
       <c r="H586">
         <f>_xlfn.XLOOKUP(E586,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="587" spans="1:8">
@@ -34204,7 +34211,7 @@
       </c>
       <c r="H587">
         <f>_xlfn.XLOOKUP(E587,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="588" spans="1:8">
@@ -34237,7 +34244,7 @@
       </c>
       <c r="H588">
         <f>_xlfn.XLOOKUP(E588,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="589" spans="1:8">
@@ -34270,7 +34277,7 @@
       </c>
       <c r="H589">
         <f>_xlfn.XLOOKUP(E589,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="590" spans="1:8">
@@ -34303,7 +34310,7 @@
       </c>
       <c r="H590">
         <f>_xlfn.XLOOKUP(E590,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="591" spans="1:8">
@@ -34336,7 +34343,7 @@
       </c>
       <c r="H591">
         <f>_xlfn.XLOOKUP(E591,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="592" spans="1:8">
@@ -34369,7 +34376,7 @@
       </c>
       <c r="H592">
         <f>_xlfn.XLOOKUP(E592,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="593" spans="1:8">
@@ -34402,7 +34409,7 @@
       </c>
       <c r="H593">
         <f>_xlfn.XLOOKUP(E593,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="594" spans="1:8">
@@ -34435,7 +34442,7 @@
       </c>
       <c r="H594">
         <f>_xlfn.XLOOKUP(E594,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="595" spans="1:8">
@@ -34468,7 +34475,7 @@
       </c>
       <c r="H595">
         <f>_xlfn.XLOOKUP(E595,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="596" spans="1:8">
@@ -35027,7 +35034,7 @@
       </c>
       <c r="H612">
         <f>_xlfn.XLOOKUP(E612,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="613" spans="1:8">
@@ -35060,7 +35067,7 @@
       </c>
       <c r="H613">
         <f>_xlfn.XLOOKUP(E613,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="614" spans="1:8">
@@ -35093,7 +35100,7 @@
       </c>
       <c r="H614">
         <f>_xlfn.XLOOKUP(E614,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="615" spans="1:8">
@@ -35126,7 +35133,7 @@
       </c>
       <c r="H615">
         <f>_xlfn.XLOOKUP(E615,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="616" spans="1:8">
@@ -35159,7 +35166,7 @@
       </c>
       <c r="H616">
         <f>_xlfn.XLOOKUP(E616,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="617" spans="1:8">
@@ -35192,7 +35199,7 @@
       </c>
       <c r="H617">
         <f>_xlfn.XLOOKUP(E617,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="618" spans="1:8">
@@ -35225,7 +35232,7 @@
       </c>
       <c r="H618">
         <f>_xlfn.XLOOKUP(E618,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="619" spans="1:8">
@@ -35258,7 +35265,7 @@
       </c>
       <c r="H619">
         <f>_xlfn.XLOOKUP(E619,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="620" spans="1:8">
@@ -35291,7 +35298,7 @@
       </c>
       <c r="H620">
         <f>_xlfn.XLOOKUP(E620,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="621" spans="1:8">
@@ -35324,7 +35331,7 @@
       </c>
       <c r="H621">
         <f>_xlfn.XLOOKUP(E621,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="622" spans="1:8">
@@ -35357,7 +35364,7 @@
       </c>
       <c r="H622">
         <f>_xlfn.XLOOKUP(E622,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="623" spans="1:8">
@@ -35390,7 +35397,7 @@
       </c>
       <c r="H623">
         <f>_xlfn.XLOOKUP(E623,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="624" spans="1:8">
@@ -35423,7 +35430,7 @@
       </c>
       <c r="H624">
         <f>_xlfn.XLOOKUP(E624,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="625" spans="1:8">
@@ -35456,7 +35463,7 @@
       </c>
       <c r="H625">
         <f>_xlfn.XLOOKUP(E625,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="626" spans="1:8">
@@ -35489,7 +35496,7 @@
       </c>
       <c r="H626">
         <f>_xlfn.XLOOKUP(E626,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="627" spans="1:8">
@@ -35522,7 +35529,7 @@
       </c>
       <c r="H627">
         <f>_xlfn.XLOOKUP(E627,SkillActive!B:B,SkillActive!K:K,,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="628" spans="1:8">
@@ -53940,7 +53947,7 @@
         <v>2</v>
       </c>
       <c r="H110" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="I110" s="7" t="s">
         <v>1583</v>
@@ -53951,11 +53958,10 @@
       <c r="K110" s="7">
         <v>1</v>
       </c>
-      <c r="L110" s="7">
-        <v>10085</v>
-      </c>
-      <c r="M110" s="7" t="s">
-        <v>234</v>
+      <c r="L110" s="7"/>
+      <c r="M110" s="7"/>
+      <c r="N110" s="7">
+        <v>2150000440</v>
       </c>
     </row>
     <row r="111" s="7" customFormat="1" ht="15.95" customHeight="1" spans="1:15">
@@ -54090,7 +54096,7 @@
         <v>2</v>
       </c>
       <c r="H114" s="7" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
       <c r="I114" s="7" t="s">
         <v>1599</v>
@@ -54101,8 +54107,11 @@
       <c r="K114" s="7">
         <v>1</v>
       </c>
-      <c r="N114" s="7">
-        <v>2150000440</v>
+      <c r="L114" s="7">
+        <v>10085</v>
+      </c>
+      <c r="M114" s="7" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="115" s="7" customFormat="1" ht="15.95" customHeight="1" spans="1:15">
@@ -58405,7 +58414,7 @@
         <v>7</v>
       </c>
       <c r="L233" s="5">
-        <v>10194</v>
+        <v>10140</v>
       </c>
       <c r="M233" s="13" t="s">
         <v>1828</v>
@@ -59902,6 +59911,9 @@
       <c r="L276" s="5">
         <v>10225</v>
       </c>
+      <c r="M276" s="5" t="s">
+        <v>329</v>
+      </c>
     </row>
     <row r="277" s="5" customFormat="1" spans="1:14">
       <c r="A277" s="4">
@@ -59971,7 +59983,7 @@
         <v>1</v>
       </c>
       <c r="L278" s="31">
-        <v>10236</v>
+        <v>10237</v>
       </c>
       <c r="M278" s="5" t="s">
         <v>329</v>
@@ -60008,10 +60020,7 @@
         <v>1</v>
       </c>
       <c r="L279" s="31">
-        <v>10237</v>
-      </c>
-      <c r="M279" s="5" t="s">
-        <v>329</v>
+        <v>10238</v>
       </c>
     </row>
     <row r="280" s="5" customFormat="1" spans="1:14">

</xml_diff>